<commit_message>
Correct reforge retention hints and show source rewards in native confirmation
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/planet_build.xlsx
+++ b/space-battleship/config_excel/planet_build.xlsx
@@ -1412,7 +1412,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>首颗星球重铸准备：达到探索条件后，派遣额外船员建设新型船坞。建成后领取设施，再选择重铸；重铸保留现有资源与永久星球奖励。</t>
+          <t>首颗星球重铸准备：达到探索条件后，派遣额外船员建设新型船坞。建成后领取设施，再选择重铸；重铸保留现有铁与铀余额与永久星球奖励。</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>首颗星球重铸准备：达到探索条件后，派遣额外船员建设新型船坞。建成后领取设施，再选择重铸；重铸保留现有资源与永久星球奖励。</t>
+          <t>首颗星球重铸准备：达到探索条件后，派遣额外船员建设新型船坞。建成后领取设施，再选择重铸；重铸保留现有铁与铀余额与永久星球奖励。</t>
         </is>
       </c>
       <c r="D8" t="n">

</xml_diff>

<commit_message>
Polish contextual drone guides and player-facing help copy
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/planet_build.xlsx
+++ b/space-battleship/config_excel/planet_build.xlsx
@@ -1412,7 +1412,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>首颗星球重铸准备：达到探索条件后，派遣额外船员建设新型船坞。建成后领取设施，再选择重铸；重铸保留现有铁与铀余额与永久星球奖励。</t>
+          <t>点「分配施工船员」开工；建好后领取船坞，再决定是否重铸。重铸前会显示保留内容和本轮重置范围。</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>首颗星球重铸准备：达到探索条件后，派遣额外船员建设新型船坞。建成后领取设施，再选择重铸；重铸保留现有铁与铀余额与永久星球奖励。</t>
+          <t>点「分配施工船员」开工；建好后领取船坞，再决定是否重铸。重铸前会显示保留内容和本轮重置范围。</t>
         </is>
       </c>
       <c r="D8" t="n">

</xml_diff>